<commit_message>
Update ROTEIROS TIMBAÚBA - 2026.xlsx
</commit_message>
<xml_diff>
--- a/base/ROTEIROS TIMBAÚBA - 2026.xlsx
+++ b/base/ROTEIROS TIMBAÚBA - 2026.xlsx
@@ -5,20 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/652cb8c1b03727a7/LOGÍSTICA/CONTRATOS/TIMBAÚBA/NOVA OPERAÇÃO/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/652cb8c1b03727a7/LOGÍSTICA/PROGRAMAÇÃO/TIMBAÚBA/tropical-timbauba-ocupacao/base/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="11_AD4D361C20488DEA4E38A050041B6F6C5ADEDD8D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{90F4AE5C-7594-4E9F-A44D-6B9B3CA2AB06}"/>
+  <xr:revisionPtr revIDLastSave="26" documentId="11_AD4D361C20488DEA4E38A050041B6F6C5ADEDD8D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA795BEE-FC28-4DB0-B56E-8230D9188BE4}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Roteiros" sheetId="2" r:id="rId1"/>
     <sheet name="Capacidade Veículos" sheetId="3" r:id="rId2"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId3"/>
-  </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Roteiros!$A$2:$H$124</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">Roteiros!$A$1:$G$124</definedName>
@@ -956,16 +953,16 @@
     <xf numFmtId="164" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -986,150 +983,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-      <xxl21:relativeUrl r:id="rId3"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Rotas - Terceiros"/>
-      <sheetName val="Roteiros"/>
-      <sheetName val="Calendário - 12x36"/>
-      <sheetName val="Rotas - Veículos"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3">
-        <row r="1">
-          <cell r="A1" t="str">
-            <v>ROTA</v>
-          </cell>
-          <cell r="B1" t="str">
-            <v>VEÍCULO</v>
-          </cell>
-        </row>
-        <row r="2">
-          <cell r="A2" t="str">
-            <v>J01</v>
-          </cell>
-          <cell r="B2">
-            <v>56</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="A3" t="str">
-            <v>J02</v>
-          </cell>
-          <cell r="B3">
-            <v>59</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="A4" t="str">
-            <v>L01</v>
-          </cell>
-          <cell r="B4">
-            <v>58</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="A5" t="str">
-            <v>L02</v>
-          </cell>
-          <cell r="B5">
-            <v>62</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="A6" t="str">
-            <v>L03</v>
-          </cell>
-          <cell r="B6">
-            <v>95</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="A7" t="str">
-            <v>L04</v>
-          </cell>
-          <cell r="B7">
-            <v>97</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="A8" t="str">
-            <v>L05</v>
-          </cell>
-          <cell r="B8">
-            <v>63</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="A9" t="str">
-            <v>N01</v>
-          </cell>
-          <cell r="B9">
-            <v>46</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="A10" t="str">
-            <v>N02</v>
-          </cell>
-          <cell r="B10">
-            <v>98</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="A11" t="str">
-            <v>P01</v>
-          </cell>
-          <cell r="B11">
-            <v>54</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="A12" t="str">
-            <v>P02</v>
-          </cell>
-          <cell r="B12">
-            <v>88</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="A13" t="str">
-            <v>P03</v>
-          </cell>
-          <cell r="B13">
-            <v>94</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="A14" t="str">
-            <v>P04</v>
-          </cell>
-          <cell r="B14">
-            <v>65</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="A15" t="str">
-            <v>P05</v>
-          </cell>
-          <cell r="B15">
-            <v>99</v>
-          </cell>
-        </row>
-      </sheetData>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1454,21 +1307,21 @@
     <col min="4" max="4" width="21.6640625" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="49.88671875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17" style="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="38.109375" style="9" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="17" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="38.21875" style="9" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="17.109375" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="105" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
@@ -1504,7 +1357,6 @@
         <v>9</v>
       </c>
       <c r="C3" s="3">
-        <f>_xlfn.XLOOKUP(B3,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>56</v>
       </c>
       <c r="D3" s="3" t="s">
@@ -1530,7 +1382,6 @@
         <v>9</v>
       </c>
       <c r="C4" s="3">
-        <f>_xlfn.XLOOKUP(B4,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>56</v>
       </c>
       <c r="D4" s="3" t="s">
@@ -1556,7 +1407,6 @@
         <v>9</v>
       </c>
       <c r="C5" s="3">
-        <f>_xlfn.XLOOKUP(B5,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>56</v>
       </c>
       <c r="D5" s="3" t="s">
@@ -1582,7 +1432,6 @@
         <v>9</v>
       </c>
       <c r="C6" s="3">
-        <f>_xlfn.XLOOKUP(B6,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>56</v>
       </c>
       <c r="D6" s="3"/>
@@ -1603,7 +1452,6 @@
         <v>9</v>
       </c>
       <c r="C7" s="3">
-        <f>_xlfn.XLOOKUP(B7,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>56</v>
       </c>
       <c r="D7" s="3"/>
@@ -1624,7 +1472,6 @@
         <v>9</v>
       </c>
       <c r="C8" s="3">
-        <f>_xlfn.XLOOKUP(B8,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>56</v>
       </c>
       <c r="D8" s="3" t="s">
@@ -1650,7 +1497,6 @@
         <v>9</v>
       </c>
       <c r="C9" s="3">
-        <f>_xlfn.XLOOKUP(B9,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>56</v>
       </c>
       <c r="D9" s="3" t="s">
@@ -1676,7 +1522,6 @@
         <v>9</v>
       </c>
       <c r="C10" s="3">
-        <f>_xlfn.XLOOKUP(B10,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>56</v>
       </c>
       <c r="D10" s="3" t="s">
@@ -1701,7 +1546,6 @@
         <v>9</v>
       </c>
       <c r="C11" s="3">
-        <f>_xlfn.XLOOKUP(B11,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>56</v>
       </c>
       <c r="D11" s="3" t="s">
@@ -1724,7 +1568,6 @@
         <v>9</v>
       </c>
       <c r="C12" s="3">
-        <f>_xlfn.XLOOKUP(B12,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>56</v>
       </c>
       <c r="D12" s="3" t="s">
@@ -1749,7 +1592,6 @@
         <v>9</v>
       </c>
       <c r="C13" s="3">
-        <f>_xlfn.XLOOKUP(B13,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>56</v>
       </c>
       <c r="D13" s="3" t="s">
@@ -1774,7 +1616,6 @@
         <v>9</v>
       </c>
       <c r="C14" s="3">
-        <f>_xlfn.XLOOKUP(B14,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>56</v>
       </c>
       <c r="D14" s="3" t="s">
@@ -1799,7 +1640,6 @@
         <v>9</v>
       </c>
       <c r="C15" s="3">
-        <f>_xlfn.XLOOKUP(B15,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>56</v>
       </c>
       <c r="D15" s="3"/>
@@ -1820,7 +1660,6 @@
         <v>9</v>
       </c>
       <c r="C16" s="3">
-        <f>_xlfn.XLOOKUP(B16,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>56</v>
       </c>
       <c r="D16" s="3" t="s">
@@ -1845,7 +1684,6 @@
         <v>9</v>
       </c>
       <c r="C17" s="3">
-        <f>_xlfn.XLOOKUP(B17,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>56</v>
       </c>
       <c r="D17" s="3" t="s">
@@ -1870,7 +1708,6 @@
         <v>9</v>
       </c>
       <c r="C18" s="3">
-        <f>_xlfn.XLOOKUP(B18,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>56</v>
       </c>
       <c r="D18" s="3"/>
@@ -1891,7 +1728,6 @@
         <v>9</v>
       </c>
       <c r="C19" s="3">
-        <f>_xlfn.XLOOKUP(B19,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>56</v>
       </c>
       <c r="D19" s="3"/>
@@ -1912,7 +1748,6 @@
         <v>29</v>
       </c>
       <c r="C20" s="3">
-        <f>_xlfn.XLOOKUP(B20,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>59</v>
       </c>
       <c r="D20" s="3"/>
@@ -1956,7 +1791,6 @@
         <v>29</v>
       </c>
       <c r="C22" s="3">
-        <f>_xlfn.XLOOKUP(B22,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>59</v>
       </c>
       <c r="D22" s="3"/>
@@ -1977,7 +1811,6 @@
         <v>29</v>
       </c>
       <c r="C23" s="3">
-        <f>_xlfn.XLOOKUP(B23,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>59</v>
       </c>
       <c r="D23" s="3"/>
@@ -2001,7 +1834,6 @@
         <v>29</v>
       </c>
       <c r="C24" s="3">
-        <f>_xlfn.XLOOKUP(B24,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>59</v>
       </c>
       <c r="D24" s="3"/>
@@ -2025,7 +1857,6 @@
         <v>29</v>
       </c>
       <c r="C25" s="3">
-        <f>_xlfn.XLOOKUP(B25,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>59</v>
       </c>
       <c r="D25" s="3"/>
@@ -2048,7 +1879,6 @@
         <v>29</v>
       </c>
       <c r="C26" s="3">
-        <f>_xlfn.XLOOKUP(B26,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>59</v>
       </c>
       <c r="D26" s="3"/>
@@ -2071,7 +1901,6 @@
         <v>29</v>
       </c>
       <c r="C27" s="3">
-        <f>_xlfn.XLOOKUP(B27,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>59</v>
       </c>
       <c r="D27" s="3"/>
@@ -2094,7 +1923,6 @@
         <v>29</v>
       </c>
       <c r="C28" s="3">
-        <f>_xlfn.XLOOKUP(B28,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>59</v>
       </c>
       <c r="D28" s="3"/>
@@ -2118,7 +1946,6 @@
         <v>29</v>
       </c>
       <c r="C29" s="3">
-        <f>_xlfn.XLOOKUP(B29,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>59</v>
       </c>
       <c r="D29" s="3"/>
@@ -2142,7 +1969,6 @@
         <v>29</v>
       </c>
       <c r="C30" s="3">
-        <f>_xlfn.XLOOKUP(B30,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>59</v>
       </c>
       <c r="D30" s="3"/>
@@ -2166,7 +1992,6 @@
         <v>29</v>
       </c>
       <c r="C31" s="3">
-        <f>_xlfn.XLOOKUP(B31,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>59</v>
       </c>
       <c r="D31" s="3"/>
@@ -2187,7 +2012,6 @@
         <v>29</v>
       </c>
       <c r="C32" s="3">
-        <f>_xlfn.XLOOKUP(B32,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>59</v>
       </c>
       <c r="D32" s="3"/>
@@ -2208,7 +2032,6 @@
         <v>29</v>
       </c>
       <c r="C33" s="3">
-        <f>_xlfn.XLOOKUP(B33,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>59</v>
       </c>
       <c r="D33" s="3"/>
@@ -2232,7 +2055,6 @@
         <v>29</v>
       </c>
       <c r="C34" s="3">
-        <f>_xlfn.XLOOKUP(B34,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>59</v>
       </c>
       <c r="D34" s="3"/>
@@ -2256,7 +2078,6 @@
         <v>29</v>
       </c>
       <c r="C35" s="3">
-        <f>_xlfn.XLOOKUP(B35,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>59</v>
       </c>
       <c r="D35" s="3"/>
@@ -2280,7 +2101,6 @@
         <v>48</v>
       </c>
       <c r="C36" s="3">
-        <f>_xlfn.XLOOKUP(B36,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>58</v>
       </c>
       <c r="D36" s="3"/>
@@ -2301,7 +2121,6 @@
         <v>48</v>
       </c>
       <c r="C37" s="3">
-        <f>_xlfn.XLOOKUP(B37,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>58</v>
       </c>
       <c r="D37" s="3"/>
@@ -2322,7 +2141,6 @@
         <v>48</v>
       </c>
       <c r="C38" s="3">
-        <f>_xlfn.XLOOKUP(B38,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>58</v>
       </c>
       <c r="D38" s="3"/>
@@ -2343,7 +2161,6 @@
         <v>48</v>
       </c>
       <c r="C39" s="3">
-        <f>_xlfn.XLOOKUP(B39,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>58</v>
       </c>
       <c r="D39" s="3"/>
@@ -2364,7 +2181,6 @@
         <v>48</v>
       </c>
       <c r="C40" s="3">
-        <f>_xlfn.XLOOKUP(B40,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>58</v>
       </c>
       <c r="D40" s="3"/>
@@ -2385,7 +2201,6 @@
         <v>48</v>
       </c>
       <c r="C41" s="3">
-        <f>_xlfn.XLOOKUP(B41,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>58</v>
       </c>
       <c r="D41" s="3"/>
@@ -2406,7 +2221,6 @@
         <v>58</v>
       </c>
       <c r="C42" s="3">
-        <f>_xlfn.XLOOKUP(B42,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>62</v>
       </c>
       <c r="D42" s="3"/>
@@ -2427,7 +2241,6 @@
         <v>58</v>
       </c>
       <c r="C43" s="3">
-        <f>_xlfn.XLOOKUP(B43,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>62</v>
       </c>
       <c r="D43" s="3"/>
@@ -2448,7 +2261,6 @@
         <v>58</v>
       </c>
       <c r="C44" s="3">
-        <f>_xlfn.XLOOKUP(B44,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>62</v>
       </c>
       <c r="D44" s="3"/>
@@ -2469,7 +2281,6 @@
         <v>58</v>
       </c>
       <c r="C45" s="3">
-        <f>_xlfn.XLOOKUP(B45,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>62</v>
       </c>
       <c r="D45" s="3"/>
@@ -2490,7 +2301,6 @@
         <v>58</v>
       </c>
       <c r="C46" s="3">
-        <f>_xlfn.XLOOKUP(B46,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>62</v>
       </c>
       <c r="D46" s="3"/>
@@ -2511,7 +2321,6 @@
         <v>64</v>
       </c>
       <c r="C47" s="3">
-        <f>_xlfn.XLOOKUP(B47,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>95</v>
       </c>
       <c r="D47" s="3"/>
@@ -2532,7 +2341,6 @@
         <v>64</v>
       </c>
       <c r="C48" s="3">
-        <f>_xlfn.XLOOKUP(B48,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>95</v>
       </c>
       <c r="D48" s="3"/>
@@ -2553,7 +2361,6 @@
         <v>64</v>
       </c>
       <c r="C49" s="3">
-        <f>_xlfn.XLOOKUP(B49,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>95</v>
       </c>
       <c r="D49" s="3"/>
@@ -2574,7 +2381,6 @@
         <v>69</v>
       </c>
       <c r="C50" s="3">
-        <f>_xlfn.XLOOKUP(B50,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>97</v>
       </c>
       <c r="D50" s="3"/>
@@ -2596,7 +2402,6 @@
         <v>69</v>
       </c>
       <c r="C51" s="3">
-        <f>_xlfn.XLOOKUP(B51,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>97</v>
       </c>
       <c r="D51" s="3"/>
@@ -2618,7 +2423,6 @@
         <v>72</v>
       </c>
       <c r="C52" s="3">
-        <f>_xlfn.XLOOKUP(B52,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>46</v>
       </c>
       <c r="D52" s="3"/>
@@ -2640,7 +2444,6 @@
         <v>72</v>
       </c>
       <c r="C53" s="3">
-        <f>_xlfn.XLOOKUP(B53,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>46</v>
       </c>
       <c r="D53" s="3"/>
@@ -2662,7 +2465,6 @@
         <v>72</v>
       </c>
       <c r="C54" s="3">
-        <f>_xlfn.XLOOKUP(B54,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>46</v>
       </c>
       <c r="D54" s="3"/>
@@ -2684,7 +2486,6 @@
         <v>72</v>
       </c>
       <c r="C55" s="3">
-        <f>_xlfn.XLOOKUP(B55,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>46</v>
       </c>
       <c r="D55" s="3"/>
@@ -2706,7 +2507,6 @@
         <v>72</v>
       </c>
       <c r="C56" s="3">
-        <f>_xlfn.XLOOKUP(B56,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>46</v>
       </c>
       <c r="D56" s="3"/>
@@ -2728,7 +2528,6 @@
         <v>72</v>
       </c>
       <c r="C57" s="3">
-        <f>_xlfn.XLOOKUP(B57,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>46</v>
       </c>
       <c r="D57" s="3"/>
@@ -2749,7 +2548,6 @@
         <v>72</v>
       </c>
       <c r="C58" s="3">
-        <f>_xlfn.XLOOKUP(B58,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>46</v>
       </c>
       <c r="D58" s="3"/>
@@ -2770,7 +2568,6 @@
         <v>72</v>
       </c>
       <c r="C59" s="3">
-        <f>_xlfn.XLOOKUP(B59,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>46</v>
       </c>
       <c r="D59" s="3"/>
@@ -2791,7 +2588,6 @@
         <v>72</v>
       </c>
       <c r="C60" s="3">
-        <f>_xlfn.XLOOKUP(B60,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>46</v>
       </c>
       <c r="D60" s="3"/>
@@ -2812,7 +2608,6 @@
         <v>72</v>
       </c>
       <c r="C61" s="3">
-        <f>_xlfn.XLOOKUP(B61,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>46</v>
       </c>
       <c r="D61" s="3"/>
@@ -2833,7 +2628,6 @@
         <v>83</v>
       </c>
       <c r="C62" s="3">
-        <f>_xlfn.XLOOKUP(B62,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>98</v>
       </c>
       <c r="D62" s="3"/>
@@ -2854,7 +2648,6 @@
         <v>83</v>
       </c>
       <c r="C63" s="3">
-        <f>_xlfn.XLOOKUP(B63,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>98</v>
       </c>
       <c r="D63" s="3"/>
@@ -2875,7 +2668,6 @@
         <v>83</v>
       </c>
       <c r="C64" s="3">
-        <f>_xlfn.XLOOKUP(B64,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>98</v>
       </c>
       <c r="D64" s="3"/>
@@ -2896,7 +2688,6 @@
         <v>83</v>
       </c>
       <c r="C65" s="3">
-        <f>_xlfn.XLOOKUP(B65,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>98</v>
       </c>
       <c r="D65" s="3"/>
@@ -2917,7 +2708,6 @@
         <v>86</v>
       </c>
       <c r="C66" s="3">
-        <f>_xlfn.XLOOKUP(B66,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>54</v>
       </c>
       <c r="D66" s="3"/>
@@ -2941,7 +2731,6 @@
         <v>86</v>
       </c>
       <c r="C67" s="3">
-        <f>_xlfn.XLOOKUP(B67,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>54</v>
       </c>
       <c r="D67" s="3"/>
@@ -2965,7 +2754,6 @@
         <v>86</v>
       </c>
       <c r="C68" s="3">
-        <f>_xlfn.XLOOKUP(B68,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>54</v>
       </c>
       <c r="D68" s="3"/>
@@ -2989,7 +2777,6 @@
         <v>86</v>
       </c>
       <c r="C69" s="3">
-        <f>_xlfn.XLOOKUP(B69,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>54</v>
       </c>
       <c r="D69" s="3"/>
@@ -3013,7 +2800,6 @@
         <v>86</v>
       </c>
       <c r="C70" s="3">
-        <f>_xlfn.XLOOKUP(B70,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>54</v>
       </c>
       <c r="D70" s="3"/>
@@ -3037,7 +2823,6 @@
         <v>86</v>
       </c>
       <c r="C71" s="3">
-        <f>_xlfn.XLOOKUP(B71,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>54</v>
       </c>
       <c r="D71" s="3"/>
@@ -3061,7 +2846,6 @@
         <v>86</v>
       </c>
       <c r="C72" s="3">
-        <f>_xlfn.XLOOKUP(B72,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>54</v>
       </c>
       <c r="D72" s="3"/>
@@ -3085,7 +2869,6 @@
         <v>86</v>
       </c>
       <c r="C73" s="3">
-        <f>_xlfn.XLOOKUP(B73,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>54</v>
       </c>
       <c r="D73" s="3"/>
@@ -3109,7 +2892,6 @@
         <v>86</v>
       </c>
       <c r="C74" s="3">
-        <f>_xlfn.XLOOKUP(B74,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>54</v>
       </c>
       <c r="D74" s="3"/>
@@ -3133,7 +2915,6 @@
         <v>86</v>
       </c>
       <c r="C75" s="3">
-        <f>_xlfn.XLOOKUP(B75,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>54</v>
       </c>
       <c r="D75" s="3"/>
@@ -3154,7 +2935,6 @@
         <v>86</v>
       </c>
       <c r="C76" s="3">
-        <f>_xlfn.XLOOKUP(B76,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>54</v>
       </c>
       <c r="D76" s="3"/>
@@ -3175,7 +2955,6 @@
         <v>86</v>
       </c>
       <c r="C77" s="3">
-        <f>_xlfn.XLOOKUP(B77,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>54</v>
       </c>
       <c r="D77" s="3"/>
@@ -3449,7 +3228,6 @@
         <v>110</v>
       </c>
       <c r="C89" s="3">
-        <f>_xlfn.XLOOKUP(B89,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>94</v>
       </c>
       <c r="D89" s="3"/>
@@ -3473,7 +3251,6 @@
         <v>110</v>
       </c>
       <c r="C90" s="3">
-        <f>_xlfn.XLOOKUP(B90,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>94</v>
       </c>
       <c r="D90" s="3"/>
@@ -3497,7 +3274,6 @@
         <v>110</v>
       </c>
       <c r="C91" s="3">
-        <f>_xlfn.XLOOKUP(B91,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>94</v>
       </c>
       <c r="D91" s="3"/>
@@ -3521,7 +3297,6 @@
         <v>110</v>
       </c>
       <c r="C92" s="3">
-        <f>_xlfn.XLOOKUP(B92,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>94</v>
       </c>
       <c r="D92" s="3"/>
@@ -3542,7 +3317,6 @@
         <v>110</v>
       </c>
       <c r="C93" s="3">
-        <f>_xlfn.XLOOKUP(B93,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>94</v>
       </c>
       <c r="D93" s="3"/>
@@ -3566,7 +3340,6 @@
         <v>110</v>
       </c>
       <c r="C94" s="3">
-        <f>_xlfn.XLOOKUP(B94,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>94</v>
       </c>
       <c r="D94" s="3"/>
@@ -3590,7 +3363,6 @@
         <v>110</v>
       </c>
       <c r="C95" s="3">
-        <f>_xlfn.XLOOKUP(B95,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>94</v>
       </c>
       <c r="D95" s="3"/>
@@ -3614,7 +3386,6 @@
         <v>110</v>
       </c>
       <c r="C96" s="3">
-        <f>_xlfn.XLOOKUP(B96,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>94</v>
       </c>
       <c r="D96" s="3"/>
@@ -3638,7 +3409,6 @@
         <v>110</v>
       </c>
       <c r="C97" s="3">
-        <f>_xlfn.XLOOKUP(B97,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>94</v>
       </c>
       <c r="D97" s="3"/>
@@ -3662,7 +3432,6 @@
         <v>110</v>
       </c>
       <c r="C98" s="3">
-        <f>_xlfn.XLOOKUP(B98,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>94</v>
       </c>
       <c r="D98" s="3"/>
@@ -3686,7 +3455,6 @@
         <v>110</v>
       </c>
       <c r="C99" s="3">
-        <f>_xlfn.XLOOKUP(B99,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>94</v>
       </c>
       <c r="D99" s="3"/>
@@ -3730,7 +3498,6 @@
         <v>110</v>
       </c>
       <c r="C101" s="3">
-        <f>_xlfn.XLOOKUP(B101,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>94</v>
       </c>
       <c r="D101" s="3"/>
@@ -3754,7 +3521,6 @@
         <v>110</v>
       </c>
       <c r="C102" s="3">
-        <f>_xlfn.XLOOKUP(B102,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>94</v>
       </c>
       <c r="D102" s="3"/>
@@ -3778,7 +3544,6 @@
         <v>110</v>
       </c>
       <c r="C103" s="3">
-        <f>_xlfn.XLOOKUP(B103,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>94</v>
       </c>
       <c r="D103" s="3"/>
@@ -3802,7 +3567,6 @@
         <v>126</v>
       </c>
       <c r="C104" s="3">
-        <f>_xlfn.XLOOKUP(B104,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>65</v>
       </c>
       <c r="D104" s="3"/>
@@ -3826,7 +3590,6 @@
         <v>126</v>
       </c>
       <c r="C105" s="3">
-        <f>_xlfn.XLOOKUP(B105,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>65</v>
       </c>
       <c r="D105" s="3"/>
@@ -3850,7 +3613,6 @@
         <v>126</v>
       </c>
       <c r="C106" s="3">
-        <f>_xlfn.XLOOKUP(B106,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>65</v>
       </c>
       <c r="D106" s="3"/>
@@ -3871,7 +3633,6 @@
         <v>126</v>
       </c>
       <c r="C107" s="3">
-        <f>_xlfn.XLOOKUP(B107,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>65</v>
       </c>
       <c r="D107" s="3"/>
@@ -3895,7 +3656,6 @@
         <v>126</v>
       </c>
       <c r="C108" s="3">
-        <f>_xlfn.XLOOKUP(B108,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>65</v>
       </c>
       <c r="D108" s="3"/>
@@ -3919,7 +3679,6 @@
         <v>126</v>
       </c>
       <c r="C109" s="3">
-        <f>_xlfn.XLOOKUP(B109,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>65</v>
       </c>
       <c r="D109" s="3"/>
@@ -3943,7 +3702,6 @@
         <v>126</v>
       </c>
       <c r="C110" s="3">
-        <f>_xlfn.XLOOKUP(B110,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>65</v>
       </c>
       <c r="D110" s="3"/>
@@ -3967,7 +3725,6 @@
         <v>126</v>
       </c>
       <c r="C111" s="3">
-        <f>_xlfn.XLOOKUP(B111,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>65</v>
       </c>
       <c r="D111" s="3"/>
@@ -3991,7 +3748,6 @@
         <v>135</v>
       </c>
       <c r="C112" s="3">
-        <f>_xlfn.XLOOKUP(B112,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>99</v>
       </c>
       <c r="D112" s="3"/>
@@ -4015,7 +3771,6 @@
         <v>135</v>
       </c>
       <c r="C113" s="3">
-        <f>_xlfn.XLOOKUP(B113,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>99</v>
       </c>
       <c r="D113" s="3"/>
@@ -4039,7 +3794,6 @@
         <v>135</v>
       </c>
       <c r="C114" s="3">
-        <f>_xlfn.XLOOKUP(B114,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>99</v>
       </c>
       <c r="D114" s="3"/>
@@ -4063,7 +3817,6 @@
         <v>135</v>
       </c>
       <c r="C115" s="3">
-        <f>_xlfn.XLOOKUP(B115,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>99</v>
       </c>
       <c r="D115" s="3"/>
@@ -4087,7 +3840,6 @@
         <v>135</v>
       </c>
       <c r="C116" s="3">
-        <f>_xlfn.XLOOKUP(B116,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>99</v>
       </c>
       <c r="D116" s="3"/>
@@ -4111,7 +3863,6 @@
         <v>135</v>
       </c>
       <c r="C117" s="3">
-        <f>_xlfn.XLOOKUP(B117,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>99</v>
       </c>
       <c r="D117" s="3"/>
@@ -4135,7 +3886,6 @@
         <v>135</v>
       </c>
       <c r="C118" s="3">
-        <f>_xlfn.XLOOKUP(B118,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>99</v>
       </c>
       <c r="D118" s="3"/>
@@ -4159,7 +3909,6 @@
         <v>135</v>
       </c>
       <c r="C119" s="3">
-        <f>_xlfn.XLOOKUP(B119,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>99</v>
       </c>
       <c r="D119" s="3"/>
@@ -4183,7 +3932,6 @@
         <v>135</v>
       </c>
       <c r="C120" s="3">
-        <f>_xlfn.XLOOKUP(B120,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>99</v>
       </c>
       <c r="D120" s="3"/>
@@ -4207,7 +3955,6 @@
         <v>135</v>
       </c>
       <c r="C121" s="3">
-        <f>_xlfn.XLOOKUP(B121,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>99</v>
       </c>
       <c r="D121" s="3"/>
@@ -4251,7 +3998,6 @@
         <v>135</v>
       </c>
       <c r="C123" s="3">
-        <f>_xlfn.XLOOKUP(B123,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>99</v>
       </c>
       <c r="D123" s="3"/>
@@ -4275,7 +4021,6 @@
         <v>135</v>
       </c>
       <c r="C124" s="3">
-        <f>_xlfn.XLOOKUP(B124,'[1]Rotas - Veículos'!$A:$A,'[1]Rotas - Veículos'!$B:$B)</f>
         <v>99</v>
       </c>
       <c r="D124" s="3"/>
@@ -4330,18 +4075,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="12" t="s">
         <v>148</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="12" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="13" t="s">
         <v>151</v>
       </c>
       <c r="B2" s="6" t="s">
@@ -4352,18 +4097,18 @@
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="14" t="s">
         <v>153</v>
       </c>
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="15" t="s">
         <v>154</v>
       </c>
-      <c r="C3" s="17">
+      <c r="C3" s="15">
         <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="13" t="s">
         <v>155</v>
       </c>
       <c r="B4" s="6" t="s">
@@ -4374,18 +4119,18 @@
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="16" t="s">
+      <c r="A5" s="14" t="s">
         <v>157</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="15" t="s">
         <v>158</v>
       </c>
-      <c r="C5" s="17">
+      <c r="C5" s="15">
         <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="15" t="s">
+      <c r="A6" s="13" t="s">
         <v>159</v>
       </c>
       <c r="B6" s="6" t="s">
@@ -4396,18 +4141,18 @@
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="16" t="s">
+      <c r="A7" s="14" t="s">
         <v>161</v>
       </c>
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="C7" s="17">
+      <c r="C7" s="15">
         <v>48</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="15" t="s">
+      <c r="A8" s="13" t="s">
         <v>163</v>
       </c>
       <c r="B8" s="6" t="s">
@@ -4418,18 +4163,18 @@
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="16" t="s">
+      <c r="A9" s="14" t="s">
         <v>165</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="15" t="s">
         <v>166</v>
       </c>
-      <c r="C9" s="17">
+      <c r="C9" s="15">
         <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="15" t="s">
+      <c r="A10" s="13" t="s">
         <v>167</v>
       </c>
       <c r="B10" s="6" t="s">
@@ -4440,18 +4185,18 @@
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="16">
+      <c r="A11" s="14">
         <v>10</v>
       </c>
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="15" t="s">
         <v>169</v>
       </c>
-      <c r="C11" s="17">
+      <c r="C11" s="15">
         <v>48</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="15">
+      <c r="A12" s="13">
         <v>11</v>
       </c>
       <c r="B12" s="6" t="s">
@@ -4462,18 +4207,18 @@
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="16">
+      <c r="A13" s="14">
         <v>12</v>
       </c>
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="15" t="s">
         <v>171</v>
       </c>
-      <c r="C13" s="17">
+      <c r="C13" s="15">
         <v>46</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="15">
+      <c r="A14" s="13">
         <v>13</v>
       </c>
       <c r="B14" s="6" t="s">
@@ -4484,18 +4229,18 @@
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="16">
+      <c r="A15" s="14">
         <v>14</v>
       </c>
-      <c r="B15" s="17" t="s">
+      <c r="B15" s="15" t="s">
         <v>173</v>
       </c>
-      <c r="C15" s="17">
+      <c r="C15" s="15">
         <v>48</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="15">
+      <c r="A16" s="13">
         <v>15</v>
       </c>
       <c r="B16" s="6" t="s">
@@ -4506,18 +4251,18 @@
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="16">
+      <c r="A17" s="14">
         <v>201</v>
       </c>
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="15" t="s">
         <v>175</v>
       </c>
-      <c r="C17" s="17">
+      <c r="C17" s="15">
         <v>48</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="15">
+      <c r="A18" s="13">
         <v>202</v>
       </c>
       <c r="B18" s="6" t="s">
@@ -4528,18 +4273,18 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="16">
+      <c r="A19" s="14">
         <v>203</v>
       </c>
-      <c r="B19" s="17" t="s">
+      <c r="B19" s="15" t="s">
         <v>177</v>
       </c>
-      <c r="C19" s="17">
+      <c r="C19" s="15">
         <v>48</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="15">
+      <c r="A20" s="13">
         <v>204</v>
       </c>
       <c r="B20" s="6" t="s">
@@ -4550,18 +4295,18 @@
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="16">
+      <c r="A21" s="14">
         <v>205</v>
       </c>
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="15" t="s">
         <v>179</v>
       </c>
-      <c r="C21" s="17">
+      <c r="C21" s="15">
         <v>48</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="15">
+      <c r="A22" s="13">
         <v>206</v>
       </c>
       <c r="B22" s="6" t="s">
@@ -4572,18 +4317,18 @@
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="16">
+      <c r="A23" s="14">
         <v>207</v>
       </c>
-      <c r="B23" s="17" t="s">
+      <c r="B23" s="15" t="s">
         <v>181</v>
       </c>
-      <c r="C23" s="17">
+      <c r="C23" s="15">
         <v>48</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="15">
+      <c r="A24" s="13">
         <v>17</v>
       </c>
       <c r="B24" s="6" t="s">
@@ -4594,18 +4339,18 @@
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="16">
+      <c r="A25" s="14">
         <v>20</v>
       </c>
-      <c r="B25" s="17" t="s">
+      <c r="B25" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="C25" s="17">
+      <c r="C25" s="15">
         <v>42</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="15">
+      <c r="A26" s="13">
         <v>23</v>
       </c>
       <c r="B26" s="6" t="s">
@@ -4616,18 +4361,18 @@
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="16">
+      <c r="A27" s="14">
         <v>24</v>
       </c>
-      <c r="B27" s="17" t="s">
+      <c r="B27" s="15" t="s">
         <v>185</v>
       </c>
-      <c r="C27" s="17">
+      <c r="C27" s="15">
         <v>44</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="15">
+      <c r="A28" s="13">
         <v>25</v>
       </c>
       <c r="B28" s="6" t="s">
@@ -4638,18 +4383,18 @@
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" s="16">
+      <c r="A29" s="14">
         <v>26</v>
       </c>
-      <c r="B29" s="17" t="s">
+      <c r="B29" s="15" t="s">
         <v>187</v>
       </c>
-      <c r="C29" s="17">
+      <c r="C29" s="15">
         <v>42</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" s="15">
+      <c r="A30" s="13">
         <v>27</v>
       </c>
       <c r="B30" s="6" t="s">
@@ -4660,18 +4405,18 @@
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31" s="16">
+      <c r="A31" s="14">
         <v>28</v>
       </c>
-      <c r="B31" s="17" t="s">
+      <c r="B31" s="15" t="s">
         <v>189</v>
       </c>
-      <c r="C31" s="17">
+      <c r="C31" s="15">
         <v>41</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A32" s="15">
+      <c r="A32" s="13">
         <v>46</v>
       </c>
       <c r="B32" s="6" t="s">
@@ -4682,18 +4427,18 @@
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A33" s="16">
+      <c r="A33" s="14">
         <v>47</v>
       </c>
-      <c r="B33" s="17" t="s">
+      <c r="B33" s="15" t="s">
         <v>191</v>
       </c>
-      <c r="C33" s="17">
+      <c r="C33" s="15">
         <v>48</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A34" s="15">
+      <c r="A34" s="13">
         <v>48</v>
       </c>
       <c r="B34" s="6" t="s">
@@ -4704,18 +4449,18 @@
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A35" s="16">
+      <c r="A35" s="14">
         <v>50</v>
       </c>
-      <c r="B35" s="17" t="s">
+      <c r="B35" s="15" t="s">
         <v>193</v>
       </c>
-      <c r="C35" s="17">
+      <c r="C35" s="15">
         <v>45</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A36" s="15">
+      <c r="A36" s="13">
         <v>51</v>
       </c>
       <c r="B36" s="6" t="s">
@@ -4726,18 +4471,18 @@
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A37" s="16">
+      <c r="A37" s="14">
         <v>52</v>
       </c>
-      <c r="B37" s="17" t="s">
+      <c r="B37" s="15" t="s">
         <v>195</v>
       </c>
-      <c r="C37" s="17">
+      <c r="C37" s="15">
         <v>45</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A38" s="15">
+      <c r="A38" s="13">
         <v>53</v>
       </c>
       <c r="B38" s="6" t="s">
@@ -4748,18 +4493,18 @@
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A39" s="16">
+      <c r="A39" s="14">
         <v>54</v>
       </c>
-      <c r="B39" s="17" t="s">
+      <c r="B39" s="15" t="s">
         <v>197</v>
       </c>
-      <c r="C39" s="17">
+      <c r="C39" s="15">
         <v>45</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A40" s="15">
+      <c r="A40" s="13">
         <v>55</v>
       </c>
       <c r="B40" s="6" t="s">
@@ -4770,18 +4515,18 @@
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A41" s="16">
+      <c r="A41" s="14">
         <v>56</v>
       </c>
-      <c r="B41" s="17" t="s">
+      <c r="B41" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="C41" s="17">
+      <c r="C41" s="15">
         <v>45</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A42" s="15">
+      <c r="A42" s="13">
         <v>57</v>
       </c>
       <c r="B42" s="6" t="s">
@@ -4792,18 +4537,18 @@
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A43" s="16">
+      <c r="A43" s="14">
         <v>58</v>
       </c>
-      <c r="B43" s="17" t="s">
+      <c r="B43" s="15" t="s">
         <v>201</v>
       </c>
-      <c r="C43" s="17">
+      <c r="C43" s="15">
         <v>45</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A44" s="15">
+      <c r="A44" s="13">
         <v>59</v>
       </c>
       <c r="B44" s="6" t="s">
@@ -4814,18 +4559,18 @@
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A45" s="16">
+      <c r="A45" s="14">
         <v>61</v>
       </c>
-      <c r="B45" s="17" t="s">
+      <c r="B45" s="15" t="s">
         <v>203</v>
       </c>
-      <c r="C45" s="17">
+      <c r="C45" s="15">
         <v>45</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A46" s="15">
+      <c r="A46" s="13">
         <v>62</v>
       </c>
       <c r="B46" s="6" t="s">
@@ -4836,18 +4581,18 @@
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A47" s="16">
+      <c r="A47" s="14">
         <v>63</v>
       </c>
-      <c r="B47" s="17" t="s">
+      <c r="B47" s="15" t="s">
         <v>205</v>
       </c>
-      <c r="C47" s="17">
+      <c r="C47" s="15">
         <v>45</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A48" s="15">
+      <c r="A48" s="13">
         <v>64</v>
       </c>
       <c r="B48" s="6" t="s">
@@ -4858,18 +4603,18 @@
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A49" s="16">
+      <c r="A49" s="14">
         <v>65</v>
       </c>
-      <c r="B49" s="17" t="s">
+      <c r="B49" s="15" t="s">
         <v>207</v>
       </c>
-      <c r="C49" s="17">
+      <c r="C49" s="15">
         <v>45</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A50" s="15">
+      <c r="A50" s="13">
         <v>81</v>
       </c>
       <c r="B50" s="6" t="s">
@@ -4880,18 +4625,18 @@
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A51" s="16">
+      <c r="A51" s="14">
         <v>83</v>
       </c>
-      <c r="B51" s="17" t="s">
+      <c r="B51" s="15" t="s">
         <v>209</v>
       </c>
-      <c r="C51" s="17">
+      <c r="C51" s="15">
         <v>45</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A52" s="15">
+      <c r="A52" s="13">
         <v>88</v>
       </c>
       <c r="B52" s="6" t="s">
@@ -4902,18 +4647,18 @@
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A53" s="16">
+      <c r="A53" s="14">
         <v>89</v>
       </c>
-      <c r="B53" s="17" t="s">
+      <c r="B53" s="15" t="s">
         <v>211</v>
       </c>
-      <c r="C53" s="17">
+      <c r="C53" s="15">
         <v>45</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A54" s="15">
+      <c r="A54" s="13">
         <v>91</v>
       </c>
       <c r="B54" s="6" t="s">
@@ -4924,18 +4669,18 @@
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A55" s="16">
+      <c r="A55" s="14">
         <v>94</v>
       </c>
-      <c r="B55" s="17" t="s">
+      <c r="B55" s="15" t="s">
         <v>213</v>
       </c>
-      <c r="C55" s="17">
+      <c r="C55" s="15">
         <v>48</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A56" s="15">
+      <c r="A56" s="13">
         <v>95</v>
       </c>
       <c r="B56" s="6" t="s">
@@ -4946,18 +4691,18 @@
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A57" s="16">
+      <c r="A57" s="14">
         <v>96</v>
       </c>
-      <c r="B57" s="17" t="s">
+      <c r="B57" s="15" t="s">
         <v>215</v>
       </c>
-      <c r="C57" s="17">
+      <c r="C57" s="15">
         <v>45</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A58" s="15">
+      <c r="A58" s="13">
         <v>97</v>
       </c>
       <c r="B58" s="6" t="s">
@@ -4968,18 +4713,18 @@
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A59" s="16">
+      <c r="A59" s="14">
         <v>98</v>
       </c>
-      <c r="B59" s="17" t="s">
+      <c r="B59" s="15" t="s">
         <v>217</v>
       </c>
-      <c r="C59" s="17">
+      <c r="C59" s="15">
         <v>48</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A60" s="15">
+      <c r="A60" s="13">
         <v>99</v>
       </c>
       <c r="B60" s="6" t="s">
@@ -4990,18 +4735,18 @@
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A61" s="16">
+      <c r="A61" s="14">
         <v>102</v>
       </c>
-      <c r="B61" s="17" t="s">
+      <c r="B61" s="15" t="s">
         <v>219</v>
       </c>
-      <c r="C61" s="17">
+      <c r="C61" s="15">
         <v>45</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A62" s="15">
+      <c r="A62" s="13">
         <v>103</v>
       </c>
       <c r="B62" s="6" t="s">
@@ -5012,18 +4757,18 @@
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A63" s="16">
+      <c r="A63" s="14">
         <v>104</v>
       </c>
-      <c r="B63" s="17" t="s">
+      <c r="B63" s="15" t="s">
         <v>221</v>
       </c>
-      <c r="C63" s="17">
+      <c r="C63" s="15">
         <v>45</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A64" s="15">
+      <c r="A64" s="13">
         <v>105</v>
       </c>
       <c r="B64" s="6" t="s">
@@ -5034,18 +4779,18 @@
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A65" s="16">
+      <c r="A65" s="14">
         <v>106</v>
       </c>
-      <c r="B65" s="17" t="s">
+      <c r="B65" s="15" t="s">
         <v>223</v>
       </c>
-      <c r="C65" s="17">
+      <c r="C65" s="15">
         <v>48</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A66" s="15">
+      <c r="A66" s="13">
         <v>107</v>
       </c>
       <c r="B66" s="6" t="s">
@@ -5056,18 +4801,18 @@
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A67" s="16">
+      <c r="A67" s="14">
         <v>108</v>
       </c>
-      <c r="B67" s="17" t="s">
+      <c r="B67" s="15" t="s">
         <v>225</v>
       </c>
-      <c r="C67" s="17">
+      <c r="C67" s="15">
         <v>48</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A68" s="15">
+      <c r="A68" s="13">
         <v>109</v>
       </c>
       <c r="B68" s="6" t="s">
@@ -5078,18 +4823,18 @@
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A69" s="16">
+      <c r="A69" s="14">
         <v>110</v>
       </c>
-      <c r="B69" s="17" t="s">
+      <c r="B69" s="15" t="s">
         <v>227</v>
       </c>
-      <c r="C69" s="17">
+      <c r="C69" s="15">
         <v>48</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A70" s="15">
+      <c r="A70" s="13">
         <v>111</v>
       </c>
       <c r="B70" s="6" t="s">
@@ -5100,18 +4845,18 @@
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A71" s="16">
+      <c r="A71" s="14">
         <v>100</v>
       </c>
-      <c r="B71" s="17" t="s">
+      <c r="B71" s="15" t="s">
         <v>229</v>
       </c>
-      <c r="C71" s="17">
+      <c r="C71" s="15">
         <v>48</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A72" s="15" t="s">
+      <c r="A72" s="13" t="s">
         <v>230</v>
       </c>
       <c r="B72" s="6"/>
@@ -5120,18 +4865,18 @@
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A73" s="16">
+      <c r="A73" s="14">
         <v>101</v>
       </c>
-      <c r="B73" s="17" t="s">
+      <c r="B73" s="15" t="s">
         <v>231</v>
       </c>
-      <c r="C73" s="17">
+      <c r="C73" s="15">
         <v>48</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A74" s="15" t="s">
+      <c r="A74" s="13" t="s">
         <v>232</v>
       </c>
       <c r="B74" s="6" t="s">
@@ -5142,18 +4887,18 @@
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A75" s="16" t="s">
+      <c r="A75" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="B75" s="17" t="s">
+      <c r="B75" s="15" t="s">
         <v>235</v>
       </c>
-      <c r="C75" s="17">
+      <c r="C75" s="15">
         <v>15</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A76" s="15" t="s">
+      <c r="A76" s="13" t="s">
         <v>236</v>
       </c>
       <c r="B76" s="6" t="s">
@@ -5164,18 +4909,18 @@
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A77" s="16" t="s">
+      <c r="A77" s="14" t="s">
         <v>238</v>
       </c>
-      <c r="B77" s="17" t="s">
+      <c r="B77" s="15" t="s">
         <v>239</v>
       </c>
-      <c r="C77" s="17">
+      <c r="C77" s="15">
         <v>15</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A78" s="15" t="s">
+      <c r="A78" s="13" t="s">
         <v>240</v>
       </c>
       <c r="B78" s="6" t="s">
@@ -5186,18 +4931,18 @@
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A79" s="16" t="s">
+      <c r="A79" s="14" t="s">
         <v>242</v>
       </c>
-      <c r="B79" s="17" t="s">
+      <c r="B79" s="15" t="s">
         <v>243</v>
       </c>
-      <c r="C79" s="17">
+      <c r="C79" s="15">
         <v>15</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A80" s="15" t="s">
+      <c r="A80" s="13" t="s">
         <v>244</v>
       </c>
       <c r="B80" s="6" t="s">
@@ -5208,18 +4953,18 @@
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A81" s="16" t="s">
+      <c r="A81" s="14" t="s">
         <v>246</v>
       </c>
-      <c r="B81" s="17" t="s">
+      <c r="B81" s="15" t="s">
         <v>247</v>
       </c>
-      <c r="C81" s="17">
+      <c r="C81" s="15">
         <v>20</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A82" s="15" t="s">
+      <c r="A82" s="13" t="s">
         <v>248</v>
       </c>
       <c r="B82" s="6" t="s">
@@ -5230,18 +4975,18 @@
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A83" s="16" t="s">
+      <c r="A83" s="14" t="s">
         <v>250</v>
       </c>
-      <c r="B83" s="17" t="s">
+      <c r="B83" s="15" t="s">
         <v>251</v>
       </c>
-      <c r="C83" s="17">
+      <c r="C83" s="15">
         <v>22</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A84" s="15" t="s">
+      <c r="A84" s="13" t="s">
         <v>252</v>
       </c>
       <c r="B84" s="6" t="s">
@@ -5252,18 +4997,18 @@
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A85" s="16" t="s">
+      <c r="A85" s="14" t="s">
         <v>254</v>
       </c>
-      <c r="B85" s="17" t="s">
+      <c r="B85" s="15" t="s">
         <v>255</v>
       </c>
-      <c r="C85" s="17">
+      <c r="C85" s="15">
         <v>28</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A86" s="15" t="s">
+      <c r="A86" s="13" t="s">
         <v>256</v>
       </c>
       <c r="B86" s="6" t="s">

</xml_diff>